<commit_message>
Update STP management and tanker features
</commit_message>
<xml_diff>
--- a/database/users.xlsx
+++ b/database/users.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J5"/>
+  <dimension ref="A1:L2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -459,10 +459,20 @@
       </c>
       <c r="I1" t="inlineStr">
         <is>
+          <t>stp_id</t>
+        </is>
+      </c>
+      <c r="J1" t="inlineStr">
+        <is>
+          <t>tanker_operator_id</t>
+        </is>
+      </c>
+      <c r="K1" t="inlineStr">
+        <is>
           <t>created_at</t>
         </is>
       </c>
-      <c r="J1" t="inlineStr">
+      <c r="L1" t="inlineStr">
         <is>
           <t>account_status</t>
         </is>
@@ -471,206 +481,52 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>USR-C06309D6C6</t>
+          <t>USR-E849398559</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Manoranjan</t>
+          <t>Gowtham</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>S</t>
+          <t>Y K</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>manoannabond</t>
+          <t>gowtham</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>7892012246</t>
+          <t>8431041386</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>mano@handsomeboi.com</t>
+          <t>eng23am0027@dsu.edu.in</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>scrypt:32768:8:1$n6DcPLzNT2NKPWIU$e71756a3355daea6b452197b48ac874d29d451a30196033817f99a6c46e878ccf41f9e5fddf286485b46e47d88ccd3203d2d8afabdfef8a1f3de6aec6d2e134c</t>
+          <t>scrypt:32768:8:1$nlszliVLEk6KUAVc$a5edeed53eb4876feb9921d66dae90eaaf42a5527e2623683e41d2f58673c29f390ffa48eadef3baf1e6b06dbb458f785c6eb66ab4abfd7a080fb98ff7096d36</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>stp</t>
-        </is>
-      </c>
-      <c r="I2" t="inlineStr">
-        <is>
-          <t>2026-08-24 16:19:42</t>
-        </is>
-      </c>
-      <c r="J2" t="inlineStr">
-        <is>
-          <t>active</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>USR-4C97A38875</t>
-        </is>
-      </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>Mohith</t>
-        </is>
-      </c>
-      <c r="C3" t="inlineStr">
-        <is>
-          <t>Mohan</t>
-        </is>
-      </c>
-      <c r="D3" t="inlineStr">
-        <is>
-          <t>mohithmohan</t>
-        </is>
-      </c>
-      <c r="E3" t="inlineStr">
-        <is>
-          <t>9845430586</t>
-        </is>
-      </c>
-      <c r="F3" t="inlineStr">
-        <is>
-          <t>mohith.mohan10102004@gmail.com</t>
-        </is>
-      </c>
-      <c r="G3" t="inlineStr">
-        <is>
-          <t>scrypt:32768:8:1$5pM2mHyrs9I1oU5U$8b4996b3f6aca158df34a98d336aaf60f3766d140ebee79130d677a240fdc6e2d611f90910ec8f40bfd3bfaed166a23d63546d94f902060357b0ac2e3262b83e</t>
-        </is>
-      </c>
-      <c r="H3" t="inlineStr">
-        <is>
-          <t>stp</t>
-        </is>
-      </c>
-      <c r="I3" t="inlineStr">
-        <is>
-          <t>2026-08-25 10:53:59</t>
-        </is>
-      </c>
-      <c r="J3" t="inlineStr">
-        <is>
-          <t>active</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>USR-6EBABEAAB7</t>
-        </is>
-      </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>Demand</t>
-        </is>
-      </c>
-      <c r="C4" t="inlineStr">
-        <is>
-          <t>Site</t>
-        </is>
-      </c>
-      <c r="D4" t="inlineStr">
-        <is>
-          <t>demandsite</t>
-        </is>
-      </c>
-      <c r="E4" t="inlineStr">
-        <is>
-          <t>9138918398</t>
-        </is>
-      </c>
-      <c r="F4" t="inlineStr">
-        <is>
-          <t>eng23am0045@dsu.edu.in</t>
-        </is>
-      </c>
-      <c r="G4" t="inlineStr">
-        <is>
-          <t>scrypt:32768:8:1$5x87t084xkZLkCj7$713ee28d5372e0cc37153f196474f45b8720e30e80d9a0081c72efa8bcb008d80c3912ee65c23e7ced684a8e1b2389c97233599c0c146d5441412b211c9525d5</t>
-        </is>
-      </c>
-      <c r="H4" t="inlineStr">
-        <is>
           <t>demand</t>
         </is>
       </c>
-      <c r="I4" t="inlineStr">
-        <is>
-          <t>2026-08-25 10:56:30</t>
-        </is>
-      </c>
-      <c r="J4" t="inlineStr">
-        <is>
-          <t>active</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>USR-ABBE84E5E3</t>
-        </is>
-      </c>
-      <c r="B5" t="inlineStr">
-        <is>
-          <t>Tanker</t>
-        </is>
-      </c>
-      <c r="C5" t="inlineStr">
-        <is>
-          <t>Site</t>
-        </is>
-      </c>
-      <c r="D5" t="inlineStr">
-        <is>
-          <t>tankersite</t>
-        </is>
-      </c>
-      <c r="E5" t="inlineStr">
-        <is>
-          <t>8249829428</t>
-        </is>
-      </c>
-      <c r="F5" t="inlineStr">
-        <is>
-          <t>xyz@gmail.com</t>
-        </is>
-      </c>
-      <c r="G5" t="inlineStr">
-        <is>
-          <t>scrypt:32768:8:1$v17oC4HMLWJBi7HL$5d362d353281fc02f6cdc9b7467d94c657db1ac478472f8215882962606733599567001034cc1c3c34184424237e756e5f6a46c34273986430e493a274fb19e3</t>
-        </is>
-      </c>
-      <c r="H5" t="inlineStr">
-        <is>
-          <t>tanker</t>
-        </is>
-      </c>
-      <c r="I5" t="inlineStr">
-        <is>
-          <t>2026-08-25 10:57:22</t>
-        </is>
-      </c>
-      <c r="J5" t="inlineStr">
+      <c r="I2" t="inlineStr"/>
+      <c r="J2" t="inlineStr"/>
+      <c r="K2" t="inlineStr">
+        <is>
+          <t>2026-08-25 16:35:38</t>
+        </is>
+      </c>
+      <c r="L2" t="inlineStr">
         <is>
           <t>active</t>
         </is>

</xml_diff>

<commit_message>
Revert "Merge pull request #6 from MohithMohan2004/gowtham-updates"
This reverts commit 0b79d8554dd07a40dc71721b51206b0c13e1a4fa, reversing
changes made to 0ff55d64ed955239686bff132a5c6c27ce85b94b.
</commit_message>
<xml_diff>
--- a/database/users.xlsx
+++ b/database/users.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L2"/>
+  <dimension ref="A1:J5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -459,20 +459,10 @@
       </c>
       <c r="I1" t="inlineStr">
         <is>
-          <t>stp_id</t>
+          <t>created_at</t>
         </is>
       </c>
       <c r="J1" t="inlineStr">
-        <is>
-          <t>tanker_operator_id</t>
-        </is>
-      </c>
-      <c r="K1" t="inlineStr">
-        <is>
-          <t>created_at</t>
-        </is>
-      </c>
-      <c r="L1" t="inlineStr">
         <is>
           <t>account_status</t>
         </is>
@@ -481,52 +471,206 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>USR-E849398559</t>
+          <t>USR-C06309D6C6</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Gowtham</t>
+          <t>Manoranjan</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Y K</t>
+          <t>S</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>gowtham</t>
+          <t>manoannabond</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>8431041386</t>
+          <t>7892012246</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>eng23am0027@dsu.edu.in</t>
+          <t>mano@handsomeboi.com</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>scrypt:32768:8:1$nlszliVLEk6KUAVc$a5edeed53eb4876feb9921d66dae90eaaf42a5527e2623683e41d2f58673c29f390ffa48eadef3baf1e6b06dbb458f785c6eb66ab4abfd7a080fb98ff7096d36</t>
+          <t>scrypt:32768:8:1$n6DcPLzNT2NKPWIU$e71756a3355daea6b452197b48ac874d29d451a30196033817f99a6c46e878ccf41f9e5fddf286485b46e47d88ccd3203d2d8afabdfef8a1f3de6aec6d2e134c</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
         <is>
+          <t>stp</t>
+        </is>
+      </c>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>2026-08-24 16:19:42</t>
+        </is>
+      </c>
+      <c r="J2" t="inlineStr">
+        <is>
+          <t>active</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>USR-4C97A38875</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Mohith</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>Mohan</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>mohithmohan</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>9845430586</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>mohith.mohan10102004@gmail.com</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>scrypt:32768:8:1$5pM2mHyrs9I1oU5U$8b4996b3f6aca158df34a98d336aaf60f3766d140ebee79130d677a240fdc6e2d611f90910ec8f40bfd3bfaed166a23d63546d94f902060357b0ac2e3262b83e</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>stp</t>
+        </is>
+      </c>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>2026-08-25 10:53:59</t>
+        </is>
+      </c>
+      <c r="J3" t="inlineStr">
+        <is>
+          <t>active</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>USR-6EBABEAAB7</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Demand</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>Site</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>demandsite</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>9138918398</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>eng23am0045@dsu.edu.in</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>scrypt:32768:8:1$5x87t084xkZLkCj7$713ee28d5372e0cc37153f196474f45b8720e30e80d9a0081c72efa8bcb008d80c3912ee65c23e7ced684a8e1b2389c97233599c0c146d5441412b211c9525d5</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
           <t>demand</t>
         </is>
       </c>
-      <c r="I2" t="inlineStr"/>
-      <c r="J2" t="inlineStr"/>
-      <c r="K2" t="inlineStr">
-        <is>
-          <t>2026-08-25 16:35:38</t>
-        </is>
-      </c>
-      <c r="L2" t="inlineStr">
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>2026-08-25 10:56:30</t>
+        </is>
+      </c>
+      <c r="J4" t="inlineStr">
+        <is>
+          <t>active</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>USR-ABBE84E5E3</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Tanker</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>Site</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>tankersite</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>8249829428</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>xyz@gmail.com</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>scrypt:32768:8:1$v17oC4HMLWJBi7HL$5d362d353281fc02f6cdc9b7467d94c657db1ac478472f8215882962606733599567001034cc1c3c34184424237e756e5f6a46c34273986430e493a274fb19e3</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>tanker</t>
+        </is>
+      </c>
+      <c r="I5" t="inlineStr">
+        <is>
+          <t>2026-08-25 10:57:22</t>
+        </is>
+      </c>
+      <c r="J5" t="inlineStr">
         <is>
           <t>active</t>
         </is>

</xml_diff>

<commit_message>
Add Gowtham integration updates
</commit_message>
<xml_diff>
--- a/database/users.xlsx
+++ b/database/users.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J5"/>
+  <dimension ref="A1:L1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -459,220 +459,22 @@
       </c>
       <c r="I1" t="inlineStr">
         <is>
+          <t>stp_id</t>
+        </is>
+      </c>
+      <c r="J1" t="inlineStr">
+        <is>
+          <t>tanker_operator_id</t>
+        </is>
+      </c>
+      <c r="K1" t="inlineStr">
+        <is>
           <t>created_at</t>
         </is>
       </c>
-      <c r="J1" t="inlineStr">
+      <c r="L1" t="inlineStr">
         <is>
           <t>account_status</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>USR-C06309D6C6</t>
-        </is>
-      </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>Manoranjan</t>
-        </is>
-      </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t>S</t>
-        </is>
-      </c>
-      <c r="D2" t="inlineStr">
-        <is>
-          <t>manoannabond</t>
-        </is>
-      </c>
-      <c r="E2" t="inlineStr">
-        <is>
-          <t>7892012246</t>
-        </is>
-      </c>
-      <c r="F2" t="inlineStr">
-        <is>
-          <t>mano@handsomeboi.com</t>
-        </is>
-      </c>
-      <c r="G2" t="inlineStr">
-        <is>
-          <t>scrypt:32768:8:1$n6DcPLzNT2NKPWIU$e71756a3355daea6b452197b48ac874d29d451a30196033817f99a6c46e878ccf41f9e5fddf286485b46e47d88ccd3203d2d8afabdfef8a1f3de6aec6d2e134c</t>
-        </is>
-      </c>
-      <c r="H2" t="inlineStr">
-        <is>
-          <t>stp</t>
-        </is>
-      </c>
-      <c r="I2" t="inlineStr">
-        <is>
-          <t>2026-08-24 16:19:42</t>
-        </is>
-      </c>
-      <c r="J2" t="inlineStr">
-        <is>
-          <t>active</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>USR-4C97A38875</t>
-        </is>
-      </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>Mohith</t>
-        </is>
-      </c>
-      <c r="C3" t="inlineStr">
-        <is>
-          <t>Mohan</t>
-        </is>
-      </c>
-      <c r="D3" t="inlineStr">
-        <is>
-          <t>mohithmohan</t>
-        </is>
-      </c>
-      <c r="E3" t="inlineStr">
-        <is>
-          <t>9845430586</t>
-        </is>
-      </c>
-      <c r="F3" t="inlineStr">
-        <is>
-          <t>mohith.mohan10102004@gmail.com</t>
-        </is>
-      </c>
-      <c r="G3" t="inlineStr">
-        <is>
-          <t>scrypt:32768:8:1$5pM2mHyrs9I1oU5U$8b4996b3f6aca158df34a98d336aaf60f3766d140ebee79130d677a240fdc6e2d611f90910ec8f40bfd3bfaed166a23d63546d94f902060357b0ac2e3262b83e</t>
-        </is>
-      </c>
-      <c r="H3" t="inlineStr">
-        <is>
-          <t>stp</t>
-        </is>
-      </c>
-      <c r="I3" t="inlineStr">
-        <is>
-          <t>2026-08-25 10:53:59</t>
-        </is>
-      </c>
-      <c r="J3" t="inlineStr">
-        <is>
-          <t>active</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>USR-6EBABEAAB7</t>
-        </is>
-      </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>Demand</t>
-        </is>
-      </c>
-      <c r="C4" t="inlineStr">
-        <is>
-          <t>Site</t>
-        </is>
-      </c>
-      <c r="D4" t="inlineStr">
-        <is>
-          <t>demandsite</t>
-        </is>
-      </c>
-      <c r="E4" t="inlineStr">
-        <is>
-          <t>9138918398</t>
-        </is>
-      </c>
-      <c r="F4" t="inlineStr">
-        <is>
-          <t>eng23am0045@dsu.edu.in</t>
-        </is>
-      </c>
-      <c r="G4" t="inlineStr">
-        <is>
-          <t>scrypt:32768:8:1$5x87t084xkZLkCj7$713ee28d5372e0cc37153f196474f45b8720e30e80d9a0081c72efa8bcb008d80c3912ee65c23e7ced684a8e1b2389c97233599c0c146d5441412b211c9525d5</t>
-        </is>
-      </c>
-      <c r="H4" t="inlineStr">
-        <is>
-          <t>demand</t>
-        </is>
-      </c>
-      <c r="I4" t="inlineStr">
-        <is>
-          <t>2026-08-25 10:56:30</t>
-        </is>
-      </c>
-      <c r="J4" t="inlineStr">
-        <is>
-          <t>active</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>USR-ABBE84E5E3</t>
-        </is>
-      </c>
-      <c r="B5" t="inlineStr">
-        <is>
-          <t>Tanker</t>
-        </is>
-      </c>
-      <c r="C5" t="inlineStr">
-        <is>
-          <t>Site</t>
-        </is>
-      </c>
-      <c r="D5" t="inlineStr">
-        <is>
-          <t>tankersite</t>
-        </is>
-      </c>
-      <c r="E5" t="inlineStr">
-        <is>
-          <t>8249829428</t>
-        </is>
-      </c>
-      <c r="F5" t="inlineStr">
-        <is>
-          <t>xyz@gmail.com</t>
-        </is>
-      </c>
-      <c r="G5" t="inlineStr">
-        <is>
-          <t>scrypt:32768:8:1$v17oC4HMLWJBi7HL$5d362d353281fc02f6cdc9b7467d94c657db1ac478472f8215882962606733599567001034cc1c3c34184424237e756e5f6a46c34273986430e493a274fb19e3</t>
-        </is>
-      </c>
-      <c r="H5" t="inlineStr">
-        <is>
-          <t>tanker</t>
-        </is>
-      </c>
-      <c r="I5" t="inlineStr">
-        <is>
-          <t>2026-08-25 10:57:22</t>
-        </is>
-      </c>
-      <c r="J5" t="inlineStr">
-        <is>
-          <t>active</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
saving current stable working project
</commit_message>
<xml_diff>
--- a/database/users.xlsx
+++ b/database/users.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L1"/>
+  <dimension ref="A1:L5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -459,22 +459,230 @@
       </c>
       <c r="I1" t="inlineStr">
         <is>
+          <t>created_at</t>
+        </is>
+      </c>
+      <c r="J1" t="inlineStr">
+        <is>
+          <t>account_status</t>
+        </is>
+      </c>
+      <c r="K1" t="inlineStr">
+        <is>
           <t>stp_id</t>
         </is>
       </c>
-      <c r="J1" t="inlineStr">
+      <c r="L1" t="inlineStr">
         <is>
           <t>tanker_operator_id</t>
         </is>
       </c>
-      <c r="K1" t="inlineStr">
-        <is>
-          <t>created_at</t>
-        </is>
-      </c>
-      <c r="L1" t="inlineStr">
-        <is>
-          <t>account_status</t>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>USR-C06309D6C6</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>Manoranjan</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>manoannabond</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>7892012246</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>mano@handsomeboi.com</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>scrypt:32768:8:1$n6DcPLzNT2NKPWIU$e71756a3355daea6b452197b48ac874d29d451a30196033817f99a6c46e878ccf41f9e5fddf286485b46e47d88ccd3203d2d8afabdfef8a1f3de6aec6d2e134c</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>stp</t>
+        </is>
+      </c>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>2026-08-24 16:19:42</t>
+        </is>
+      </c>
+      <c r="J2" t="inlineStr">
+        <is>
+          <t>active</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>USR-4C97A38875</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Mohith</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>Mohan</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>mohithmohan</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>9845430586</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>mohith.mohan10102004@gmail.com</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>scrypt:32768:8:1$5pM2mHyrs9I1oU5U$8b4996b3f6aca158df34a98d336aaf60f3766d140ebee79130d677a240fdc6e2d611f90910ec8f40bfd3bfaed166a23d63546d94f902060357b0ac2e3262b83e</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>stp</t>
+        </is>
+      </c>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>2026-08-25 10:53:59</t>
+        </is>
+      </c>
+      <c r="J3" t="inlineStr">
+        <is>
+          <t>active</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>USR-6EBABEAAB7</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Demand</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>Site</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>demandsite</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>9138918398</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>eng23am0045@dsu.edu.in</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>scrypt:32768:8:1$5x87t084xkZLkCj7$713ee28d5372e0cc37153f196474f45b8720e30e80d9a0081c72efa8bcb008d80c3912ee65c23e7ced684a8e1b2389c97233599c0c146d5441412b211c9525d5</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>demand</t>
+        </is>
+      </c>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>2026-08-25 10:56:30</t>
+        </is>
+      </c>
+      <c r="J4" t="inlineStr">
+        <is>
+          <t>active</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>USR-ABBE84E5E3</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Tanker</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>Site</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>tankersite</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>8249829428</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>xyz@gmail.com</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>scrypt:32768:8:1$v17oC4HMLWJBi7HL$5d362d353281fc02f6cdc9b7467d94c657db1ac478472f8215882962606733599567001034cc1c3c34184424237e756e5f6a46c34273986430e493a274fb19e3</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>tanker</t>
+        </is>
+      </c>
+      <c r="I5" t="inlineStr">
+        <is>
+          <t>2026-08-25 10:57:22</t>
+        </is>
+      </c>
+      <c r="J5" t="inlineStr">
+        <is>
+          <t>active</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
fixed request water pipeline errors
</commit_message>
<xml_diff>
--- a/database/users.xlsx
+++ b/database/users.xlsx
@@ -4,26 +4,41 @@
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
     <sheet name="Users" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
-  <calcPr calcId="124519" fullCalcOnLoad="1"/>
+  <calcPr calcId="124519" fullCalcOnLoad="1" refMode="A1" iterate="0" iterateCount="100" iterateDelta="0.0001"/>
 </workbook>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="1">
+  <fonts count="4">
     <font>
       <name val="Calibri"/>
+      <charset val="1"/>
       <family val="2"/>
       <color theme="1"/>
       <sz val="11"/>
-      <scheme val="minor"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <family val="0"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <family val="0"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <family val="0"/>
+      <sz val="10"/>
     </font>
   </fonts>
   <fills count="2">
@@ -43,16 +58,33 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="1">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+  <cellStyleXfs count="6">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1">
+      <alignment horizontal="general" vertical="bottom"/>
+    </xf>
+    <xf numFmtId="43" fontId="3" fillId="0" borderId="0"/>
+    <xf numFmtId="41" fontId="3" fillId="0" borderId="0"/>
+    <xf numFmtId="44" fontId="3" fillId="0" borderId="0"/>
+    <xf numFmtId="42" fontId="3" fillId="0" borderId="0"/>
+    <xf numFmtId="9" fontId="3" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="3">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="general" vertical="bottom"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="general" vertical="bottom"/>
+    </xf>
   </cellXfs>
-  <cellStyles count="1">
-    <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
+  <cellStyles count="6">
+    <cellStyle name="Normal" xfId="0" builtinId="0"/>
+    <cellStyle name="Comma" xfId="1" builtinId="3"/>
+    <cellStyle name="Comma [0]" xfId="2" builtinId="6"/>
+    <cellStyle name="Currency" xfId="3" builtinId="4"/>
+    <cellStyle name="Currency [0]" xfId="4" builtinId="7"/>
+    <cellStyle name="Percent" xfId="5" builtinId="5"/>
   </cellStyles>
-  <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
   <colors>
     <indexedColors>
       <rgbColor rgb="00000000"/>
@@ -125,41 +157,41 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Office Theme">
   <a:themeElements>
     <a:clrScheme name="Office">
       <a:dk1>
-        <a:sysClr val="windowText" lastClr="000000"/>
+        <a:srgbClr val="000000"/>
       </a:dk1>
       <a:lt1>
-        <a:sysClr val="window" lastClr="FFFFFF"/>
+        <a:srgbClr val="ffffff"/>
       </a:lt1>
       <a:dk2>
-        <a:srgbClr val="1F497D"/>
+        <a:srgbClr val="1f497d"/>
       </a:dk2>
       <a:lt2>
-        <a:srgbClr val="EEECE1"/>
+        <a:srgbClr val="eeece1"/>
       </a:lt2>
       <a:accent1>
-        <a:srgbClr val="4F81BD"/>
+        <a:srgbClr val="4f81bd"/>
       </a:accent1>
       <a:accent2>
-        <a:srgbClr val="C0504D"/>
+        <a:srgbClr val="c0504d"/>
       </a:accent2>
       <a:accent3>
-        <a:srgbClr val="9BBB59"/>
+        <a:srgbClr val="9bbb59"/>
       </a:accent3>
       <a:accent4>
-        <a:srgbClr val="8064A2"/>
+        <a:srgbClr val="8064a2"/>
       </a:accent4>
       <a:accent5>
-        <a:srgbClr val="4BACC6"/>
+        <a:srgbClr val="4bacc6"/>
       </a:accent5>
       <a:accent6>
-        <a:srgbClr val="F79646"/>
+        <a:srgbClr val="f79646"/>
       </a:accent6>
       <a:hlink>
-        <a:srgbClr val="0000FF"/>
+        <a:srgbClr val="0000ff"/>
       </a:hlink>
       <a:folHlink>
         <a:srgbClr val="800080"/>
@@ -167,312 +199,204 @@
     </a:clrScheme>
     <a:fontScheme name="Office">
       <a:majorFont>
-        <a:latin typeface="Cambria"/>
+        <a:latin typeface="Cambria" pitchFamily="0" charset="1"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
-        <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
-        <a:font script="Hang" typeface="맑은 고딕"/>
-        <a:font script="Hans" typeface="宋体"/>
-        <a:font script="Hant" typeface="新細明體"/>
-        <a:font script="Arab" typeface="Times New Roman"/>
-        <a:font script="Hebr" typeface="Times New Roman"/>
-        <a:font script="Thai" typeface="Tahoma"/>
-        <a:font script="Ethi" typeface="Nyala"/>
-        <a:font script="Beng" typeface="Vrinda"/>
-        <a:font script="Gujr" typeface="Shruti"/>
-        <a:font script="Khmr" typeface="MoolBoran"/>
-        <a:font script="Knda" typeface="Tunga"/>
-        <a:font script="Guru" typeface="Raavi"/>
-        <a:font script="Cans" typeface="Euphemia"/>
-        <a:font script="Cher" typeface="Plantagenet Cherokee"/>
-        <a:font script="Yiii" typeface="Microsoft Yi Baiti"/>
-        <a:font script="Tibt" typeface="Microsoft Himalaya"/>
-        <a:font script="Thaa" typeface="MV Boli"/>
-        <a:font script="Deva" typeface="Mangal"/>
-        <a:font script="Telu" typeface="Gautami"/>
-        <a:font script="Taml" typeface="Latha"/>
-        <a:font script="Syrc" typeface="Estrangelo Edessa"/>
-        <a:font script="Orya" typeface="Kalinga"/>
-        <a:font script="Mlym" typeface="Kartika"/>
-        <a:font script="Laoo" typeface="DokChampa"/>
-        <a:font script="Sinh" typeface="Iskoola Pota"/>
-        <a:font script="Mong" typeface="Mongolian Baiti"/>
-        <a:font script="Viet" typeface="Times New Roman"/>
-        <a:font script="Uigh" typeface="Microsoft Uighur"/>
       </a:majorFont>
       <a:minorFont>
-        <a:latin typeface="Calibri"/>
+        <a:latin typeface="Calibri" pitchFamily="0" charset="1"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
-        <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
-        <a:font script="Hang" typeface="맑은 고딕"/>
-        <a:font script="Hans" typeface="宋体"/>
-        <a:font script="Hant" typeface="新細明體"/>
-        <a:font script="Arab" typeface="Arial"/>
-        <a:font script="Hebr" typeface="Arial"/>
-        <a:font script="Thai" typeface="Tahoma"/>
-        <a:font script="Ethi" typeface="Nyala"/>
-        <a:font script="Beng" typeface="Vrinda"/>
-        <a:font script="Gujr" typeface="Shruti"/>
-        <a:font script="Khmr" typeface="DaunPenh"/>
-        <a:font script="Knda" typeface="Tunga"/>
-        <a:font script="Guru" typeface="Raavi"/>
-        <a:font script="Cans" typeface="Euphemia"/>
-        <a:font script="Cher" typeface="Plantagenet Cherokee"/>
-        <a:font script="Yiii" typeface="Microsoft Yi Baiti"/>
-        <a:font script="Tibt" typeface="Microsoft Himalaya"/>
-        <a:font script="Thaa" typeface="MV Boli"/>
-        <a:font script="Deva" typeface="Mangal"/>
-        <a:font script="Telu" typeface="Gautami"/>
-        <a:font script="Taml" typeface="Latha"/>
-        <a:font script="Syrc" typeface="Estrangelo Edessa"/>
-        <a:font script="Orya" typeface="Kalinga"/>
-        <a:font script="Mlym" typeface="Kartika"/>
-        <a:font script="Laoo" typeface="DokChampa"/>
-        <a:font script="Sinh" typeface="Iskoola Pota"/>
-        <a:font script="Mong" typeface="Mongolian Baiti"/>
-        <a:font script="Viet" typeface="Arial"/>
-        <a:font script="Uigh" typeface="Microsoft Uighur"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office">
+    <a:fmtScheme>
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
         </a:solidFill>
-        <a:gradFill rotWithShape="1">
+        <a:gradFill>
           <a:gsLst>
             <a:gs pos="0">
               <a:schemeClr val="phClr">
                 <a:tint val="50000"/>
-                <a:satMod val="300000"/>
               </a:schemeClr>
             </a:gs>
             <a:gs pos="35000">
               <a:schemeClr val="phClr">
                 <a:tint val="37000"/>
-                <a:satMod val="300000"/>
               </a:schemeClr>
             </a:gs>
             <a:gs pos="100000">
               <a:schemeClr val="phClr">
                 <a:tint val="15000"/>
-                <a:satMod val="350000"/>
               </a:schemeClr>
             </a:gs>
           </a:gsLst>
           <a:lin ang="16200000" scaled="1"/>
+          <a:tileRect l="0" t="0" r="0" b="0"/>
         </a:gradFill>
-        <a:gradFill rotWithShape="1">
+        <a:gradFill>
           <a:gsLst>
             <a:gs pos="0">
               <a:schemeClr val="phClr">
                 <a:shade val="51000"/>
-                <a:satMod val="130000"/>
               </a:schemeClr>
             </a:gs>
             <a:gs pos="80000">
               <a:schemeClr val="phClr">
                 <a:shade val="93000"/>
-                <a:satMod val="130000"/>
               </a:schemeClr>
             </a:gs>
             <a:gs pos="100000">
               <a:schemeClr val="phClr">
                 <a:shade val="94000"/>
-                <a:satMod val="135000"/>
               </a:schemeClr>
             </a:gs>
           </a:gsLst>
           <a:lin ang="16200000" scaled="0"/>
+          <a:tileRect l="0" t="0" r="0" b="0"/>
         </a:gradFill>
       </a:fillStyleLst>
       <a:lnStyleLst>
         <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
-          <a:solidFill>
-            <a:schemeClr val="phClr">
-              <a:shade val="95000"/>
-              <a:satMod val="105000"/>
-            </a:schemeClr>
-          </a:solidFill>
           <a:prstDash val="solid"/>
         </a:ln>
         <a:ln w="25400" cap="flat" cmpd="sng" algn="ctr">
-          <a:solidFill>
-            <a:schemeClr val="phClr"/>
-          </a:solidFill>
           <a:prstDash val="solid"/>
         </a:ln>
         <a:ln w="38100" cap="flat" cmpd="sng" algn="ctr">
-          <a:solidFill>
-            <a:schemeClr val="phClr"/>
-          </a:solidFill>
           <a:prstDash val="solid"/>
         </a:ln>
       </a:lnStyleLst>
       <a:effectStyleLst>
         <a:effectStyle>
-          <a:effectLst>
-            <a:outerShdw blurRad="40000" dist="20000" dir="5400000" rotWithShape="0">
-              <a:srgbClr val="000000">
-                <a:alpha val="38000"/>
-              </a:srgbClr>
-            </a:outerShdw>
-          </a:effectLst>
+          <a:effectLst/>
         </a:effectStyle>
         <a:effectStyle>
-          <a:effectLst>
-            <a:outerShdw blurRad="40000" dist="23000" dir="5400000" rotWithShape="0">
-              <a:srgbClr val="000000">
-                <a:alpha val="35000"/>
-              </a:srgbClr>
-            </a:outerShdw>
-          </a:effectLst>
+          <a:effectLst/>
         </a:effectStyle>
         <a:effectStyle>
-          <a:effectLst>
-            <a:outerShdw blurRad="40000" dist="23000" dir="5400000" rotWithShape="0">
-              <a:srgbClr val="000000">
-                <a:alpha val="35000"/>
-              </a:srgbClr>
-            </a:outerShdw>
-          </a:effectLst>
-          <a:scene3d>
-            <a:camera prst="orthographicFront">
-              <a:rot lat="0" lon="0" rev="0"/>
-            </a:camera>
-            <a:lightRig rig="threePt" dir="t">
-              <a:rot lat="0" lon="0" rev="1200000"/>
-            </a:lightRig>
-          </a:scene3d>
-          <a:sp3d>
-            <a:bevelT w="63500" h="25400"/>
-          </a:sp3d>
+          <a:effectLst/>
         </a:effectStyle>
       </a:effectStyleLst>
       <a:bgFillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
         </a:solidFill>
-        <a:gradFill rotWithShape="1">
+        <a:gradFill>
           <a:gsLst>
             <a:gs pos="0">
               <a:schemeClr val="phClr">
                 <a:tint val="40000"/>
-                <a:satMod val="350000"/>
               </a:schemeClr>
             </a:gs>
             <a:gs pos="40000">
               <a:schemeClr val="phClr">
                 <a:tint val="45000"/>
                 <a:shade val="99000"/>
-                <a:satMod val="350000"/>
               </a:schemeClr>
             </a:gs>
             <a:gs pos="100000">
               <a:schemeClr val="phClr">
                 <a:shade val="20000"/>
-                <a:satMod val="255000"/>
               </a:schemeClr>
             </a:gs>
           </a:gsLst>
           <a:path path="circle">
             <a:fillToRect l="50000" t="-80000" r="50000" b="180000"/>
           </a:path>
+          <a:tileRect l="0" t="0" r="0" b="0"/>
         </a:gradFill>
-        <a:gradFill rotWithShape="1">
+        <a:gradFill>
           <a:gsLst>
             <a:gs pos="0">
               <a:schemeClr val="phClr">
                 <a:tint val="80000"/>
-                <a:satMod val="300000"/>
               </a:schemeClr>
             </a:gs>
             <a:gs pos="100000">
               <a:schemeClr val="phClr">
                 <a:shade val="30000"/>
-                <a:satMod val="200000"/>
               </a:schemeClr>
             </a:gs>
           </a:gsLst>
           <a:path path="circle">
             <a:fillToRect l="50000" t="50000" r="50000" b="50000"/>
           </a:path>
+          <a:tileRect l="0" t="0" r="0" b="0"/>
         </a:gradFill>
       </a:bgFillStyleLst>
     </a:fmtScheme>
   </a:themeElements>
-  <a:objectDefaults/>
-  <a:extraClrSchemeLst/>
 </a:theme>
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
+  <sheetPr filterMode="0">
     <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
+    <pageSetUpPr fitToPage="0"/>
   </sheetPr>
   <dimension ref="A1:L2"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="8" defaultColWidth="8.59765625" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
   <sheetData>
-    <row r="1">
-      <c r="A1" t="inlineStr">
+    <row r="1" ht="15" customHeight="1" s="1">
+      <c r="A1" s="2" t="inlineStr">
         <is>
           <t>user_id</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="2" t="inlineStr">
         <is>
           <t>first_name</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="C1" s="2" t="inlineStr">
         <is>
           <t>last_name</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="D1" s="2" t="inlineStr">
         <is>
           <t>username</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="E1" s="2" t="inlineStr">
         <is>
           <t>mobile</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="F1" s="2" t="inlineStr">
         <is>
           <t>email</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
+      <c r="G1" s="2" t="inlineStr">
         <is>
           <t>password_hash</t>
         </is>
       </c>
-      <c r="H1" t="inlineStr">
+      <c r="H1" s="2" t="inlineStr">
         <is>
           <t>role</t>
         </is>
       </c>
-      <c r="I1" t="inlineStr">
+      <c r="I1" s="2" t="inlineStr">
         <is>
           <t>stp_id</t>
         </is>
       </c>
-      <c r="J1" t="inlineStr">
+      <c r="J1" s="2" t="inlineStr">
         <is>
           <t>tanker_operator_id</t>
         </is>
       </c>
-      <c r="K1" t="inlineStr">
+      <c r="K1" s="2" t="inlineStr">
         <is>
           <t>created_at</t>
         </is>
       </c>
-      <c r="L1" t="inlineStr">
+      <c r="L1" s="2" t="inlineStr">
         <is>
           <t>account_status</t>
         </is>
@@ -481,7 +405,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>USR-431F029C6D</t>
+          <t>USR-1D13054C22</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -496,7 +420,7 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>manoss</t>
+          <t>demandop</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
@@ -506,28 +430,24 @@
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>mohith.mohan@outlook.com</t>
+          <t>mohith.mohan10102004@gmail.com</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>scrypt:32768:8:1$3YA7M3Vx95ZRFo5o$395e2a950dd87bcdee8401c78d271aaedefd8152dd867e39190791dce1276a5688302dd584462ffbbd36983bf5d2e058055fb6bbb6380e93e8fdb667e61684c6</t>
+          <t>scrypt:32768:8:1$Z0nmBUpQGmHEvstj$ca0d7343c459fe90f7dc08e6608ef8e9c15c008b225515e8eef6dfe7244358b48d6ec0759d5dc0f377c4fdbca27c0e25ddc170c3d2d00af5f41b4e5c97cd56e6</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>stp</t>
-        </is>
-      </c>
-      <c r="I2" t="inlineStr">
-        <is>
-          <t>PSTP008</t>
-        </is>
-      </c>
+          <t>demand</t>
+        </is>
+      </c>
+      <c r="I2" t="inlineStr"/>
       <c r="J2" t="inlineStr"/>
       <c r="K2" t="inlineStr">
         <is>
-          <t>2026-09-01 10:09:51</t>
+          <t>2026-09-06 18:21:44</t>
         </is>
       </c>
       <c r="L2" t="inlineStr">
@@ -537,6 +457,8 @@
       </c>
     </row>
   </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <printOptions horizontalCentered="0" verticalCentered="0" headings="0" gridLines="0" gridLinesSet="1"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
+  <pageSetup orientation="portrait" paperSize="9" scale="100" fitToHeight="1" fitToWidth="1" pageOrder="downThenOver" blackAndWhite="0" draft="0" horizontalDpi="300" verticalDpi="300" copies="1"/>
 </worksheet>
 </file>
</xml_diff>